<commit_message>
Refactor test results and update assertions
- Updated test results in `test_backend_live.json`, `test_backend_llm_failures.json`, and `test_ui_frontend.json` to reflect new execution times and outputs.
- Changed the status of several tests from "Fail" to "Pass" based on recent fixes.
- Adjusted evidence and actual messages in test results for clarity and accuracy.
- Enhanced error handling in `test_BE_005_unrecognised_auth_mode_fails_closed` to capture server startup issues more effectively.
- Modified assertions in `test_BE_058_rate_limit_spoofed_forwarded_for` to include lockout status in the recorded output.
- Updated secret detection logic in `test_BE_053_no_hardcoded_secrets` to include additional file types and improve clarity in output.
- Refined the test for malformed upstream responses in `test_BE_065_malformed_upstream_follows_documented_contract` to simplify error reporting.
- Added fixes documentation in `catalog.py` for clarity on recent changes and their implications.
</commit_message>
<xml_diff>
--- a/qa/test_report.xlsx
+++ b/qa/test_report.xlsx
@@ -14,8 +14,8 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Cases'!$A$1:$J$102</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Defects'!$A$1:$H$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Not Tested &amp; Out of Scope'!$A$1:$E$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Defects'!$A$1:$J$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Not Tested &amp; Out of Scope'!$A$1:$E$25</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -525,7 +525,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24 10:29</t>
+          <t>2026-10-24 10:50</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>02f4fcc Document the demo deployment</t>
+          <t>9bfcf95 Add comprehensive tests for backend LLM failures and UI interactions</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,15 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>M README.md</t>
+          <t>M .env.example
+ M Code/backend/chatbot/auth.py
+ M Code/backend/chatbot/config.py
+ M Code/backend/chatbot/llm.py
+ M Code/backend/chatbot/main.py
+ M Code/backend/chatbot/search.py
+ M Code/backend/tests/test_auth.py
+ M Code/frontend/app.js
+ M Documents/configuration.md</t>
         </is>
       </c>
     </row>
@@ -1092,7 +1100,7 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>54 of 57 Critical/High tests passed. 0 Critical/High failed and 3 are Blocked (they need a live Azure OpenAI model: context recall, grounding quality, prompt-injection resistance), so the 'Works as expected' rule (all Critical and High must pass) is not met. The core chat flow, validation, error handling, auth gate, uploads, XSS protection, responsiveness and accessibility all work in local/mock mode. 7 lower-priority tests failed, giving 7 defects (4 Medium, 3 Low): token not revoked on logout, rate limit/lockout bypass via X-Forwarded-For, sign-in turned off by an AUTH_MODE typo, and a typed question lost while waiting.</t>
+          <t>54 of 57 Critical/High tests passed; 0 Critical/High failed and 3 are Blocked (they need a live Azure OpenAI model: context recall, grounding quality, prompt-injection resistance), so the rule 'all Critical and High must pass' for 'Works as expected' is not met. 0 tests failed in total. Defects: 7 found, 7 fixed and verified by re-test, 0 open. The chat flow, validation, error handling, sign-in, uploads, XSS protection, responsiveness and accessibility all work in local/mock mode.</t>
         </is>
       </c>
     </row>
@@ -1207,7 +1215,7 @@
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>exit 0: 109 passed in 6.00s</t>
+          <t>exit 0: 109 passed in 4.62s</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
@@ -1267,7 +1275,7 @@
       <c r="I3" s="4" t="inlineStr">
         <is>
           <t>$ .venv/bin/python -m pytest 'qa/tests/test_backend_live.py::test_BE_002_starts_with_documented_config'  → exit 0
-cd Code/backend &amp;&amp; RATE_LIMIT_PER_MINUTE=0 .venv/bin/python -m uvicorn chatbot.main:app --port 53861</t>
+cd Code/backend &amp;&amp; RATE_LIMIT_PER_MINUTE=0 .venv/bin/python -m uvicorn chatbot.main:app --port 42007</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr"/>
@@ -1316,7 +1324,7 @@
       <c r="I4" s="4" t="inlineStr">
         <is>
           <t>$ .venv/bin/python -m pytest 'qa/tests/test_backend_live.py::test_BE_003_azure_mode_missing_settings'  → exit 0
-cd Code/backend &amp;&amp; CHATBOT_MODE=azure .venv/bin/python -m uvicorn chatbot.main:app --port 49911</t>
+cd Code/backend &amp;&amp; CHATBOT_MODE=azure .venv/bin/python -m uvicorn chatbot.main:app --port 47897</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr"/>
@@ -1365,7 +1373,7 @@
       <c r="I5" s="4" t="inlineStr">
         <is>
           <t>$ .venv/bin/python -m pytest 'qa/tests/test_backend_live.py::test_BE_004_invalid_config_values'  → exit 0
-cd Code/backend &amp;&amp; CHATBOT_MODE=bogus RATE_LIMIT_PER_MINUTE=abc MAX_UPLOAD_MB=lots SEARCH_TOP_K=-5 MAX_HISTORY_TURNS=x ALLOW_DOCUMENT_UPLOAD=maybe .venv/bin/python -m uvicorn chatbot.main:app --port 40667</t>
+cd Code/backend &amp;&amp; CHATBOT_MODE=bogus RATE_LIMIT_PER_MINUTE=abc MAX_UPLOAD_MB=lots SEARCH_TOP_K=-5 MAX_HISTORY_TURNS=x ALLOW_DOCUMENT_UPLOAD=maybe .venv/bin/python -m uvicorn chatbot.main:app --port 54151</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr"/>
@@ -1403,19 +1411,18 @@
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>started=True; authMode reported='pasword'; unauthenticated chat=200; GET / = 200 (chat page and API open without sign-in, Sign out button hidden)
-Assertion: AssertionError: AUTH_MODE typo silently disables sign-in (fails open)</t>
+          <t>app refused to start: exit code=1; RuntimeError: AUTH_MODE must be 'none' or 'password', not 'pasword'</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>$ .venv/bin/python -m pytest 'qa/tests/test_backend_live.py::test_BE_005_unrecognised_auth_mode_fails_closed'  → exit 1
-cd Code/backend &amp;&amp; AUTH_MODE=pasword DEMO_PASSWORD=&lt;test-value&gt; .venv/bin/python -m uvicorn chatbot.main:app --port 33043</t>
+          <t>$ .venv/bin/python -m pytest 'qa/tests/test_backend_live.py::test_BE_005_unrecognised_auth_mode_fails_closed'  → exit 0
+cd Code/backend &amp;&amp; AUTH_MODE=pasword DEMO_PASSWORD=&lt;test-value&gt; .venv/bin/python -m uvicorn chatbot.main:app --port 58489</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
@@ -2564,18 +2571,17 @@
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>logout 200; chat after logout (cookie dropped) 401; replay of pre-logout cookie -&gt; 200
-Assertion: AssertionError: token still valid after logout (no server-side revocation)</t>
+          <t>logout 200; chat after logout (cookie dropped) 401; replay of pre-logout cookie -&gt; 401</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>$ .venv/bin/python -m pytest 'qa/tests/test_backend_api.py::test_BE_029_logout_revokes_session'  → exit 1</t>
+          <t>$ .venv/bin/python -m pytest 'qa/tests/test_backend_api.py::test_BE_029_logout_revokes_session'  → exit 0</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
@@ -2665,7 +2671,7 @@
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>502 {"error":{"code":"upstream_error","message":"The service could not answer right now. Please try again shortly."}} in 0.07s</t>
+          <t>502 {"error":{"code":"upstream_error","message":"The service could not answer right now. Please try again shortly."}} in 0.06s</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr">
@@ -2858,7 +2864,7 @@
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>non-JSON body -&gt; 500 {"error":{"code":"internal_error","message":"Something went wrong. Please try again."}} in 0.02s | JSON without choices -&gt; 500 {"error":{"code":"internal_error","message":"Something went wrong. Please try again."}} in 0.01s | empty choices -&gt; 500 {"error":{"code":"internal_error","message":"Something went wrong. Please try again."}} in 0.01s | truncated JSON -&gt; 500 {"error":{"code":"internal_error","message":"Something went wrong. Please try again."}} in 0.02s</t>
+          <t>non-JSON body -&gt; 502 {"error":{"code":"upstream_error","message":"The service could not answer right now. Please try again shortly."}} in 0.00s | JSON without choices -&gt; 502 {"error":{"code":"upstream_error","message":"The service could not answer right now. Please try again shortly."}} in 0.00s | empty choices -&gt; 502 {"error":{"code":"upstream_error","message":"The service could not answer right now. Please try again shortly."}} in 0.00s | truncated JSON -&gt; 500 {"error":{"code":"internal_error","message":"Something went wrong. Please try again."}} in 0.01s</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr">
@@ -2954,7 +2960,7 @@
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
-          <t>production client timeout=60.0, max_retries=2; non-responding LLM -&gt; UpstreamError (HTTP 502) after 181.5s (3 connection attempts). Front end fetch has no timeout, so the user waits this long.</t>
+          <t>production client timeout=60.0, max_retries=2; non-responding LLM -&gt; UpstreamError (HTTP 502) after 181.6s (3 connection attempts). Front end fetch has no timeout, so the user waits this long.</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr">
@@ -3002,7 +3008,7 @@
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t>search 500 -&gt; 502 {"error":{"code":"upstream_error","message":"The service could not answer right now. Please try again shortly."}} in 0.00s | search 503 -&gt; 503 {"error":{"code":"busy","message":"Azure AI Search is busy. Try again in a moment."}} in 0.00s | search 429 -&gt; 503 {"error":{"code":"busy","message":"Azure AI Search is busy. Try again in a moment."}} in 0.00s | search 403 -&gt; 502 {"error":{"code":"upstream_error","message":"The service could not answer right now. Please try again shortly."}} in 0.00s | search timeout -&gt; 502 {"error":{"code":"upstream_error","message":"The service could not answer right now. Please try again shortly."}} in 0.00s</t>
+          <t>search 500 -&gt; 502 {"error":{"code":"upstream_error","message":"The service could not answer right now. Please try again shortly."}} in 0.01s | search 503 -&gt; 503 {"error":{"code":"busy","message":"Azure AI Search is busy. Try again in a moment."}} in 0.01s | search 429 -&gt; 503 {"error":{"code":"busy","message":"Azure AI Search is busy. Try again in a moment."}} in 0.01s | search 403 -&gt; 502 {"error":{"code":"upstream_error","message":"The service could not answer right now. Please try again shortly."}} in 0.00s | search timeout -&gt; 502 {"error":{"code":"upstream_error","message":"The service could not answer right now. Please try again shortly."}} in 0.00s</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr">
@@ -3674,7 +3680,7 @@
       </c>
       <c r="G53" s="4" t="inlineStr">
         <is>
-          <t>chat 200; sensitive strings found in server logs: 0; example log line: ['2026-10-24 10:25:34,644 INFO chatbot.service: Answered a question: 2 history messages, 2 sources, 2 cited']</t>
+          <t>chat 200; sensitive strings found in server logs: 0; example log line: ['2026-10-24 10:43:32,636 INFO chatbot.service: Answered a question: 2 history messages, 2 sources, 2 cited']</t>
         </is>
       </c>
       <c r="H53" s="4" t="inlineStr">
@@ -3722,7 +3728,7 @@
       </c>
       <c r="G54" s="4" t="inlineStr">
         <is>
-          <t>83 tracked files scanned; matches outside unit tests: []; matches in unit-test fixtures (dummy values): [('Code/backend/tests/test_api.py', 61), ('Code/backend/tests/test_auth.py', 21), ('Code/backend/tests/test_auth.py', 40), ('Code/backend/tests/test_auth.py', 54), ('Code/backend/tests/test_auth.py', 63), ('Code/backend/tests/test_search.py', 147), ('Code/backend/tests/test_search.py', 148)]</t>
+          <t>106 tracked files scanned; matches outside unit tests: []; matches in unit-test fixtures (dummy values): [('Code/backend/tests/test_api.py', 61), ('Code/backend/tests/test_auth.py', 21), ('Code/backend/tests/test_auth.py', 40), ('Code/backend/tests/test_auth.py', 54), ('Code/backend/tests/test_auth.py', 63), ('Code/backend/tests/test_search.py', 147), ('Code/backend/tests/test_search.py', 148), ('qa/evidence/junit.xml', 52), ('qa/tests/test_backend_api.py', 212), ('qa/tests/test_backend_api.py', 228), ('qa/tests/test_backend_api.py', 230), ('qa/tests/test_backend_api.py', 241), ('qa/tests/test_backend_api.py', 260), ('qa/tests/test_backend_api.py', 261), ('qa/tests/test_backend_api.py', 264), ('qa/tests/test_backend_api.py', 265), ('qa/tests/test_backend_api.py', 277), ('qa/tests/test_backend_api.py', 278), ('qa/tests/test_backend_api.py', 291), ('qa/tests/test_backend_api.py', 299), ('qa/tests/test_backend_api.py', 418), ('qa/tests/test_backend_api.py', 418), ('qa/tests/test_backend_api.py', 452), ('qa/tests/test_backend_live.py', 63), ('qa/tests/test_backend_live.py', 88), ('qa/tests/test_backend_llm_failures.py', 21), ('qa/tests/test_backend_llm_failures.py', 129)]</t>
         </is>
       </c>
       <c r="H54" s="4" t="inlineStr">
@@ -3818,7 +3824,7 @@
       </c>
       <c r="G56" s="4" t="inlineStr">
         <is>
-          <t>12 sequential requests (mock LLM): median 2.6 ms, max 11.2 ms</t>
+          <t>12 sequential requests (mock LLM): median 3.5 ms, max 7.4 ms</t>
         </is>
       </c>
       <c r="H56" s="4" t="inlineStr">
@@ -3866,7 +3872,7 @@
       </c>
       <c r="G57" s="4" t="inlineStr">
         <is>
-          <t>10 simultaneous: statuses [200], all answered=True, wall 0.25s, slowest 0.24s | 50 simultaneous: statuses [200], all answered=True, wall 1.01s, slowest 0.86s</t>
+          <t>10 simultaneous: statuses [200], all answered=True, wall 0.21s, slowest 0.20s | 50 simultaneous: statuses [200], all answered=True, wall 1.09s, slowest 0.98s</t>
         </is>
       </c>
       <c r="H57" s="4" t="inlineStr">
@@ -3962,18 +3968,17 @@
       </c>
       <c r="G59" s="4" t="inlineStr">
         <is>
-          <t>30 chats from one client with rotating X-Forwarded-For -&gt; 0x429; 12 wrong logins rotating XFF -&gt; 0x429 (lockout never triggered)
-Assertion: AssertionError: per-IP rate limit bypassed by a client-supplied X-Forwarded-For header</t>
+          <t>30 chats from one client with rotating X-Forwarded-For -&gt; 10x429; 12 wrong logins rotating XFF -&gt; 7x429 (lockout triggered)</t>
         </is>
       </c>
       <c r="H59" s="4" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I59" s="4" t="inlineStr">
         <is>
-          <t>$ .venv/bin/python -m pytest 'qa/tests/test_backend_api.py::test_BE_058_rate_limit_spoofed_forwarded_for'  → exit 1</t>
+          <t>$ .venv/bin/python -m pytest 'qa/tests/test_backend_api.py::test_BE_058_rate_limit_spoofed_forwarded_for'  → exit 0</t>
         </is>
       </c>
       <c r="J59" s="4" t="inlineStr">
@@ -4171,7 +4176,7 @@
       <c r="I63" s="4" t="inlineStr">
         <is>
           <t>$ .venv/bin/python -m pytest 'qa/tests/test_backend_live.py::test_BE_062_docker_image'  → exit 0
-docker build -t qa-ai-based-chatbot:test . &amp;&amp; docker run -p 48933:8000 qa-ai-based-chatbot:test</t>
+docker build -t qa-ai-based-chatbot:test . &amp;&amp; docker run -p 38809:8000 qa-ai-based-chatbot:test</t>
         </is>
       </c>
       <c r="J63" s="4" t="inlineStr"/>
@@ -4305,18 +4310,17 @@
       </c>
       <c r="G66" s="4" t="inlineStr">
         <is>
-          <t>LLM reply with empty choices -&gt; 500 internal_error; AI Search 200 with non-JSON body -&gt; 500 internal_error (server log shows an 'Unhandled error' traceback)
-Assertion: assert (500, 500) == (502, 502)</t>
+          <t>LLM reply with empty choices -&gt; 502 upstream_error; AI Search 200 with non-JSON body -&gt; 502 upstream_error</t>
         </is>
       </c>
       <c r="H66" s="4" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I66" s="4" t="inlineStr">
         <is>
-          <t>$ .venv/bin/python -m pytest 'qa/tests/test_backend_llm_failures.py::test_BE_065_malformed_upstream_follows_documented_contract'  → exit 1</t>
+          <t>$ .venv/bin/python -m pytest 'qa/tests/test_backend_llm_failures.py::test_BE_065_malformed_upstream_follows_documented_contract'  → exit 0</t>
         </is>
       </c>
       <c r="J66" s="4" t="inlineStr">
@@ -5270,18 +5274,17 @@
       </c>
       <c r="G86" s="4" t="inlineStr">
         <is>
-          <t>input box right after Enter=''; requests sent=['What does the warranty cover?']; user messages shown=['What does the warranty cover?']; second question anywhere (screen/request/input)=False
-Assertion: AssertionError: second question silently discarded: input cleared but ask() returned early because busy</t>
+          <t>input box right after Enter='And how do I return a product?'; requests sent=['What does the warranty cover?']; user messages shown=['What does the warranty cover?']; second question anywhere (screen/request/input)=True</t>
         </is>
       </c>
       <c r="H86" s="4" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I86" s="4" t="inlineStr">
         <is>
-          <t>$ .venv/bin/python -m pytest 'qa/tests/test_ui_frontend.py::test_UI_021_question_typed_while_waiting_is_not_lost'  → exit 1</t>
+          <t>$ .venv/bin/python -m pytest 'qa/tests/test_ui_frontend.py::test_UI_021_question_typed_while_waiting_is_not_lost'  → exit 0</t>
         </is>
       </c>
       <c r="J86" s="4" t="inlineStr">
@@ -5371,18 +5374,17 @@
       </c>
       <c r="G88" s="4" t="inlineStr">
         <is>
-          <t>previous answer length=9299 chars; follow-up result: error='history.1.content: String should have at most 8000 characters'; bot replies=1
-Assertion: AssertionError: a long previous answer makes every follow-up fail (history content &gt; 8000 chars -&gt; 422)</t>
+          <t>previous answer length=9299 chars; follow-up result: error=''; bot replies=2</t>
         </is>
       </c>
       <c r="H88" s="4" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I88" s="4" t="inlineStr">
         <is>
-          <t>$ .venv/bin/python -m pytest 'qa/tests/test_ui_frontend.py::test_UI_023_follow_up_after_very_long_answer'  → exit 1</t>
+          <t>$ .venv/bin/python -m pytest 'qa/tests/test_ui_frontend.py::test_UI_023_follow_up_after_very_long_answer'  → exit 0</t>
         </is>
       </c>
       <c r="J88" s="4" t="inlineStr">
@@ -6048,18 +6050,17 @@
       </c>
       <c r="G102" s="4" t="inlineStr">
         <is>
-          <t>sessionStorage keys=['chatbot.uploadKey']; upload key stored in clear text=True
-Assertion: AssertionError: upload key persisted in sessionStorage</t>
+          <t>sessionStorage keys=[]; upload key stored in clear text=False</t>
         </is>
       </c>
       <c r="H102" s="4" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I102" s="4" t="inlineStr">
         <is>
-          <t>$ .venv/bin/python -m pytest 'qa/tests/test_ui_frontend.py::test_FE_014_no_secret_in_session_storage'  → exit 1</t>
+          <t>$ .venv/bin/python -m pytest 'qa/tests/test_ui_frontend.py::test_FE_014_no_secret_in_session_storage'  → exit 0</t>
         </is>
       </c>
       <c r="J102" s="4" t="inlineStr">
@@ -6099,7 +6100,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -6109,7 +6110,9 @@
     <col width="50" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="70" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6140,7 +6143,7 @@
       </c>
       <c r="F1" s="5" t="inlineStr">
         <is>
-          <t>Expected vs Actual</t>
+          <t>Expected vs Actual (first run)</t>
         </is>
       </c>
       <c r="G1" s="5" t="inlineStr">
@@ -6150,7 +6153,17 @@
       </c>
       <c r="H1" s="5" t="inlineStr">
         <is>
-          <t>Likely cause (analysis only)</t>
+          <t>Likely cause</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>Fix applied</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>Status</t>
         </is>
       </c>
     </row>
@@ -6196,6 +6209,16 @@
           <t>auth.py issues a stateless `expiry.HMAC` token; /api/logout only deletes the cookie in the browser. No server-side revocation (denylist/session version).</t>
         </is>
       </c>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>auth.py: each sign-in token carries a random nonce (`expiry.nonce.signature`) and /api/logout revokes it on the server (in memory). Limit: the revocation list is per worker/instance, so with several workers a copied token stays valid on the others until it expires.</t>
+        </is>
+      </c>
+      <c r="J2" s="4" t="inlineStr">
+        <is>
+          <t>Fixed – verified by re-test</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -6239,6 +6262,16 @@
           <t>main.py client_ip() trusts the first X-Forwarded-For entry from any caller. Local runs and Docker are affected. On App Service it depends on whether the front end overwrites or appends to that header; if it appends, production is affected too.</t>
         </is>
       </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>main.py client_ip(): X-Forwarded-For is ignored unless TRUST_FORWARDED_FOR is true (default true only on App Service, where WEBSITE_SITE_NAME is set), and then only the last, proxy-added entry is used.</t>
+        </is>
+      </c>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>Fixed – verified by re-test</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -6282,6 +6315,16 @@
           <t>main.py builds the password gate only when auth_mode == 'password'; config.py does not check AUTH_MODE against the allowed values. The ARM template uses a dropdown, so the risk is mainly manual or .env setups.</t>
         </is>
       </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>main.py create_app(): AUTH_MODE other than 'none'/'password' raises a RuntimeError at startup (fails closed).</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>Fixed – verified by re-test</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -6325,6 +6368,16 @@
           <t>app.js submit handler clears the textarea before calling ask(); ask() returns early when busy. Only the Send button is disabled, so Enter still submits.</t>
         </is>
       </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>app.js: the submit handler returns before clearing the box while an answer is loading, so the next question stays in the input.</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>Fixed – verified by re-test</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -6368,6 +6421,16 @@
           <t>main.py ChatMessage.content max_length=8000, but app.js resends full previous answers as history. CHAT_MAX_TOKENS=2000 makes such answers rare but possible. The raw validation text is shown to the user.</t>
         </is>
       </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>app.js: each history entry sent to the API is cut to 8,000 characters (the API's limit).</t>
+        </is>
+      </c>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>Fixed – verified by re-test</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -6411,6 +6474,16 @@
           <t>llm.py reads response.choices[0] outside the try/except; search.py calls response.json() without catching JSON errors.</t>
         </is>
       </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>llm.py: an unexpected response shape raises UpstreamError; search.py: non-JSON/non-object replies raise UpstreamError (both → 502 upstream_error).</t>
+        </is>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>Fixed – verified by re-test</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -6454,9 +6527,19 @@
           <t>app.js stores the key with storage.set(KEY_KEY, …) for convenience. Exposure is limited by the strict CSP (script-src 'self') and tab scope.</t>
         </is>
       </c>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>app.js: the upload key is kept in a JavaScript variable only; any key stored by an earlier version is removed from sessionStorage on load.</t>
+        </is>
+      </c>
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t>Fixed – verified by re-test</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H8"/>
+  <autoFilter ref="A1:J8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6467,7 +6550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -6905,7 +6988,7 @@
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>A hung LLM is cut off after ~181 s (60 s timeout × 3 attempts). The UI has no request timeout or Stop button, so the user waits that long (BE-037).</t>
+          <t>Sign-out revocation (DEF-01 fix) is held in memory per worker; the Docker image runs 2 gunicorn workers, so a copied token could still work on the other worker until expiry. A shared store would be needed for full revocation.</t>
         </is>
       </c>
     </row>
@@ -6932,7 +7015,7 @@
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Local (mock) mode only matches ASCII words, so every non-English question gets 'not found' (BE-015). Live AI Search is not affected.</t>
+          <t>Fixing the failed tests changed app code: Code/backend/chatbot/{auth,main,config,llm,search}.py, Code/frontend/app.js, Documents/configuration.md, .env.example, and one assertion in Code/backend/tests/test_auth.py (token format now has three parts).</t>
         </is>
       </c>
     </row>
@@ -6959,7 +7042,7 @@
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>The local keyword retriever matches some off-topic questions to unrelated passages (e.g. a bomb question returned the warranty-claim sentence). It quotes text and never generates any, so this is harmless (BE-051).</t>
+          <t>A hung LLM is cut off after ~181 s (60 s timeout × 3 attempts). The UI has no request timeout or Stop button, so the user waits that long (BE-037).</t>
         </is>
       </c>
     </row>
@@ -6986,7 +7069,7 @@
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>Invalid numeric settings (e.g. RATE_LIMIT_PER_MINUTE=abc) silently fall back to defaults without a log warning (BE-004).</t>
+          <t>Local (mock) mode only matches ASCII words, so every non-English question gets 'not found' (BE-015). Live AI Search is not affected.</t>
         </is>
       </c>
     </row>
@@ -7013,7 +7096,7 @@
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>Validation messages can be cryptic, e.g. '16: JSON decode error' (the number is a character offset) (BE-016).</t>
+          <t>The local keyword retriever matches some off-topic questions to unrelated passages (e.g. a bomb question returned the warranty-claim sentence). It quotes text and never generates any, so this is harmless (BE-051).</t>
         </is>
       </c>
     </row>
@@ -7040,7 +7123,7 @@
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>No HSTS header from the app. App Service is set to httpsOnly with TLS 1.2 in the template, so this is acceptable.</t>
+          <t>Invalid numeric settings (e.g. RATE_LIMIT_PER_MINUTE=abc) silently fall back to defaults without a log warning (BE-004).</t>
         </is>
       </c>
     </row>
@@ -7067,7 +7150,7 @@
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>axe moderate (not serious) findings: 'region' (composer/footnote outside landmarks) and 'heading-order' (h3 'Sources' under h1) (FE-010).</t>
+          <t>Validation messages can be cryptic, e.g. '16: JSON decode error' (the number is a character offset) (BE-016).</t>
         </is>
       </c>
     </row>
@@ -7094,12 +7177,66 @@
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
+          <t>No HSTS header from the app. App Service is set to httpsOnly with TLS 1.2 in the template, so this is acceptable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Observation</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>axe moderate (not serious) findings: 'region' (composer/footnote outside landmarks) and 'heading-order' (h3 'Sources' under h1) (FE-010).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Observation</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
           <t>The textarea's own outline is removed; its focus indicator is the composer border changing to the brand colour (FE-011).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E23"/>
+  <autoFilter ref="A1:E25"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>